<commit_message>
draft for rq2 results - task-agent coupling, along with more data analysis and plots
</commit_message>
<xml_diff>
--- a/figures/rq2/agent-harness-distribution.xlsx
+++ b/figures/rq2/agent-harness-distribution.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Code\STG\what-are-they-doing\figures\rq2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{9A6DA58F-DB5B-4C37-B6F3-DF26C20A0836}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FE1ECD0-98C6-42E8-9A75-8D6EFE29EA24}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-24789" yWindow="5743" windowWidth="24892" windowHeight="15634" xr2:uid="{A9BDEA09-76A8-4D12-A73E-92A55D0F5EBD}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="19380" windowHeight="21690" xr2:uid="{A9BDEA09-76A8-4D12-A73E-92A55D0F5EBD}"/>
   </bookViews>
   <sheets>
     <sheet name="agent-harness-distribution" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1852,25 +1865,25 @@
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{02D57815-91ED-43cb-92C2-25804820EDAC}">
                   <c15:fullRef>
-                    <c15:sqref>'agent-harness-distribution'!$B$3:$AB$3</c15:sqref>
+                    <c15:sqref>'agent-harness-distribution'!$B$4:$AB$4</c15:sqref>
                   </c15:fullRef>
                 </c:ext>
               </c:extLst>
-              <c:f>('agent-harness-distribution'!$D$3,'agent-harness-distribution'!$F$3,'agent-harness-distribution'!$H$3,'agent-harness-distribution'!$J$3,'agent-harness-distribution'!$L$3,'agent-harness-distribution'!$N$3,'agent-harness-distribution'!$P$3,'agent-harness-distribution'!$R$3,'agent-harness-distribution'!$T$3,'agent-harness-distribution'!$V$3,'agent-harness-distribution'!$X$3,'agent-harness-distribution'!$Z$3,'agent-harness-distribution'!$AB$3)</c:f>
+              <c:f>('agent-harness-distribution'!$D$4,'agent-harness-distribution'!$F$4,'agent-harness-distribution'!$H$4,'agent-harness-distribution'!$J$4,'agent-harness-distribution'!$L$4,'agent-harness-distribution'!$N$4,'agent-harness-distribution'!$P$4,'agent-harness-distribution'!$R$4,'agent-harness-distribution'!$T$4,'agent-harness-distribution'!$V$4,'agent-harness-distribution'!$X$4,'agent-harness-distribution'!$Z$4,'agent-harness-distribution'!$AB$4)</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0.1</c:v>
+                  <c:v>0.4</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>23.6</c:v>
+                  <c:v>33.799999999999997</c:v>
                 </c:pt>
                 <c:pt idx="2">
+                  <c:v>2.6</c:v>
+                </c:pt>
+                <c:pt idx="3">
                   <c:v>0</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>4</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0</c:v>
@@ -1879,19 +1892,19 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0</c:v>
+                  <c:v>0.1</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.6</c:v>
+                  <c:v>1.9</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>70.599999999999994</c:v>
+                  <c:v>60.1</c:v>
                 </c:pt>
                 <c:pt idx="9">
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>1.1000000000000001</c:v>
                 </c:pt>
                 <c:pt idx="11">
                   <c:v>0</c:v>
@@ -9613,37 +9626,37 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8F3648BA-EB12-4499-BBC7-2F12F24248E1}" name="Table1" displayName="Table1" ref="A1:AB10" totalsRowShown="0" headerRowDxfId="0" dataDxfId="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8F3648BA-EB12-4499-BBC7-2F12F24248E1}" name="Table1" displayName="Table1" ref="A1:AB10" totalsRowShown="0" headerRowDxfId="15" dataDxfId="14">
   <autoFilter ref="A1:AB10" xr:uid="{8F3648BA-EB12-4499-BBC7-2F12F24248E1}"/>
   <tableColumns count="28">
-    <tableColumn id="1" xr3:uid="{EA98B5FC-DC33-48A5-8307-774B475EE246}" name="developer" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{EA98B5FC-DC33-48A5-8307-774B475EE246}" name="developer" dataDxfId="13"/>
     <tableColumn id="2" xr3:uid="{8C8992C9-94FA-49D1-BE12-89F5223B46CC}" name="commits_total"/>
     <tableColumn id="3" xr3:uid="{00FC5F10-DCA5-4255-97A9-63D21EFDBE76}" name="amp_count"/>
-    <tableColumn id="4" xr3:uid="{59C54ED2-62E1-4730-9211-12C32DB8BA6E}" name="amp_pct" dataDxfId="14"/>
+    <tableColumn id="4" xr3:uid="{59C54ED2-62E1-4730-9211-12C32DB8BA6E}" name="amp_pct" dataDxfId="12"/>
     <tableColumn id="5" xr3:uid="{1F0382D4-D4AE-44B6-BF51-DA2AB694AA84}" name="claude_code_count"/>
-    <tableColumn id="6" xr3:uid="{7368E15C-3F52-4C59-BE78-65FEFC896AF8}" name="claude_code_pct" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{7368E15C-3F52-4C59-BE78-65FEFC896AF8}" name="claude_code_pct" dataDxfId="11"/>
     <tableColumn id="7" xr3:uid="{041AD0D4-A81C-441F-89CE-42B518FF4BFA}" name="codex_count"/>
-    <tableColumn id="8" xr3:uid="{0E3336A8-0138-4BFC-9E0B-C2EF23220995}" name="codex_pct" dataDxfId="12"/>
+    <tableColumn id="8" xr3:uid="{0E3336A8-0138-4BFC-9E0B-C2EF23220995}" name="codex_pct" dataDxfId="10"/>
     <tableColumn id="9" xr3:uid="{F8300DDB-AB41-49A0-9121-C0FD4EBE5D60}" name="copilot_count"/>
-    <tableColumn id="10" xr3:uid="{79507842-D5B4-4C1B-9387-E61029405B0E}" name="copilot_pct" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{79507842-D5B4-4C1B-9387-E61029405B0E}" name="copilot_pct" dataDxfId="9"/>
     <tableColumn id="11" xr3:uid="{5DDD0807-6CB1-471E-8CE1-7600FF16586A}" name="cursor_count"/>
-    <tableColumn id="12" xr3:uid="{0A8214D9-B66D-4AAC-A4C3-7F1E87996FB0}" name="cursor_pct" dataDxfId="10"/>
+    <tableColumn id="12" xr3:uid="{0A8214D9-B66D-4AAC-A4C3-7F1E87996FB0}" name="cursor_pct" dataDxfId="8"/>
     <tableColumn id="13" xr3:uid="{DE041210-9A03-4DA3-9667-D5787EFAFAA1}" name="gastown_count"/>
-    <tableColumn id="14" xr3:uid="{D52FF272-2687-42E8-84D9-F2AF83FB32BC}" name="gastown_pct" dataDxfId="9"/>
+    <tableColumn id="14" xr3:uid="{D52FF272-2687-42E8-84D9-F2AF83FB32BC}" name="gastown_pct" dataDxfId="7"/>
     <tableColumn id="15" xr3:uid="{19467E7D-16CB-4C94-8810-A37794BD9C83}" name="gemini_count"/>
-    <tableColumn id="16" xr3:uid="{601F3672-DFE8-4529-BB7F-62A7B3CE6CB3}" name="gemini_pct" dataDxfId="8"/>
+    <tableColumn id="16" xr3:uid="{601F3672-DFE8-4529-BB7F-62A7B3CE6CB3}" name="gemini_pct" dataDxfId="6"/>
     <tableColumn id="17" xr3:uid="{F4390A90-7576-4A86-98F5-E921C85D79E7}" name="multi_agent_count"/>
-    <tableColumn id="18" xr3:uid="{2712CF2D-BE46-49B1-A2DF-EFE7E0FC15E2}" name="multi_agent_pct" dataDxfId="7"/>
+    <tableColumn id="18" xr3:uid="{2712CF2D-BE46-49B1-A2DF-EFE7E0FC15E2}" name="multi_agent_pct" dataDxfId="5"/>
     <tableColumn id="19" xr3:uid="{230D7396-62E4-4AEB-B3F1-F7072A605010}" name="no_signal_count"/>
-    <tableColumn id="20" xr3:uid="{702BFEC8-9A72-43DC-9319-D8E5FEB93A05}" name="no_signal_pct" dataDxfId="6"/>
+    <tableColumn id="20" xr3:uid="{702BFEC8-9A72-43DC-9319-D8E5FEB93A05}" name="no_signal_pct" dataDxfId="4"/>
     <tableColumn id="21" xr3:uid="{2CDFA2EB-D627-4A33-8347-81AD333B7E90}" name="opencode_count"/>
-    <tableColumn id="22" xr3:uid="{C59328C9-271F-488B-8FD9-C30810B6B3C5}" name="opencode_pct" dataDxfId="5"/>
+    <tableColumn id="22" xr3:uid="{C59328C9-271F-488B-8FD9-C30810B6B3C5}" name="opencode_pct" dataDxfId="3"/>
     <tableColumn id="23" xr3:uid="{E38CF4B0-15DB-4555-8313-33C268E428D2}" name="pi_count"/>
-    <tableColumn id="24" xr3:uid="{8D37F7A8-D273-4B9F-BAC1-C580A1FB5AE8}" name="pi_pct" dataDxfId="4"/>
+    <tableColumn id="24" xr3:uid="{8D37F7A8-D273-4B9F-BAC1-C580A1FB5AE8}" name="pi_pct" dataDxfId="2"/>
     <tableColumn id="25" xr3:uid="{EDE2C98E-88A3-45CF-A9BE-A06DAB9EFDFD}" name="qwen_code_count"/>
-    <tableColumn id="26" xr3:uid="{D655CC36-0479-4FE9-83BB-2E9173FDF5B6}" name="qwen_code_pct" dataDxfId="3"/>
+    <tableColumn id="26" xr3:uid="{D655CC36-0479-4FE9-83BB-2E9173FDF5B6}" name="qwen_code_pct" dataDxfId="1"/>
     <tableColumn id="27" xr3:uid="{941E7770-715E-4504-B45F-53A8E2817A03}" name="windsurf_count"/>
-    <tableColumn id="28" xr3:uid="{EF353681-8376-4E44-B80B-E73FE53CF4CD}" name="windsurf_pct" dataDxfId="2"/>
+    <tableColumn id="28" xr3:uid="{EF353681-8376-4E44-B80B-E73FE53CF4CD}" name="windsurf_pct" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>